<commit_message>
grid anaysis done, changed PMHT to MHT, added cluster analysis
</commit_message>
<xml_diff>
--- a/data/PKD7_HT.xlsx
+++ b/data/PKD7_HT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Studia\Master\master_thesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F513A2C-C53D-4337-96B5-A5634A0B74C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70719935-4DBE-4B2B-90E7-9BDC28282B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{325C4884-A6C6-409C-AA77-3BDB61C1E2FA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1310" uniqueCount="663">
   <si>
     <t>O</t>
   </si>
@@ -1098,9 +1098,6 @@
   </si>
   <si>
     <t>3600Z</t>
-  </si>
-  <si>
-    <t>PMHT</t>
   </si>
   <si>
     <t>3530Z</t>
@@ -2515,15 +2512,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>0</v>
@@ -2531,7 +2528,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>0</v>
@@ -2539,7 +2536,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>0</v>
@@ -2547,7 +2544,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>0</v>
@@ -2555,7 +2552,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>0</v>
@@ -2563,7 +2560,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>0</v>
@@ -2571,7 +2568,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>0</v>
@@ -2579,7 +2576,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>0</v>
@@ -2587,7 +2584,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>0</v>
@@ -2595,7 +2592,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>0</v>
@@ -2603,7 +2600,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>0</v>
@@ -2611,7 +2608,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>0</v>
@@ -2619,7 +2616,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>0</v>
@@ -2627,7 +2624,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>0</v>
@@ -2635,7 +2632,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>0</v>
@@ -2643,7 +2640,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>0</v>
@@ -2651,7 +2648,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>0</v>
@@ -2659,7 +2656,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>0</v>
@@ -2667,7 +2664,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>0</v>
@@ -2675,7 +2672,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>0</v>
@@ -2683,7 +2680,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>0</v>
@@ -2691,7 +2688,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>0</v>
@@ -2699,7 +2696,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>0</v>
@@ -2707,7 +2704,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>0</v>
@@ -2715,7 +2712,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>0</v>
@@ -2723,7 +2720,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>0</v>
@@ -2731,7 +2728,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>0</v>
@@ -2739,7 +2736,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>0</v>
@@ -2747,7 +2744,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>0</v>
@@ -2755,7 +2752,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>0</v>
@@ -2763,7 +2760,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>0</v>
@@ -2771,7 +2768,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>0</v>
@@ -2779,7 +2776,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>0</v>
@@ -2787,7 +2784,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>0</v>
@@ -2795,7 +2792,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>0</v>
@@ -2803,7 +2800,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>0</v>
@@ -2811,7 +2808,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>0</v>
@@ -2819,7 +2816,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>0</v>
@@ -2827,7 +2824,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>0</v>
@@ -2835,7 +2832,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>0</v>
@@ -2843,7 +2840,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>0</v>
@@ -2851,7 +2848,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>0</v>
@@ -2859,7 +2856,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>0</v>
@@ -2867,7 +2864,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>0</v>
@@ -2875,7 +2872,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>0</v>
@@ -2883,7 +2880,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>0</v>
@@ -2891,7 +2888,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>0</v>
@@ -2899,7 +2896,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>0</v>
@@ -2907,7 +2904,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>0</v>
@@ -2915,7 +2912,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>0</v>
@@ -2923,7 +2920,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>0</v>
@@ -2931,7 +2928,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>0</v>
@@ -2939,7 +2936,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>0</v>
@@ -2947,7 +2944,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>0</v>
@@ -2955,623 +2952,623 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" s="6" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" s="6" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97" s="6" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" s="6" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A105" s="6" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107" s="6" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109" s="6" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A111" s="6" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" s="6" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" s="6" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117" s="6" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119" s="6" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" s="4" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121" s="6" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" s="6" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A124" s="4" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" s="6" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A126" s="4" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A127" s="6" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A128" s="4" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A130" s="4" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A131" s="6" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A132" s="4" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A133" s="6" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B133" s="5" t="s">
         <v>16</v>
@@ -3579,7 +3576,7 @@
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A134" s="4" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>16</v>
@@ -3587,7 +3584,7 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A135" s="6" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>16</v>
@@ -3595,151 +3592,151 @@
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A136" s="4" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A137" s="6" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A138" s="4" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A139" s="6" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A140" s="4" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A141" s="6" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A142" s="4" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A143" s="6" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A144" s="4" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A145" s="6" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A146" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A147" s="6" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A148" s="4" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A149" s="6" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A150" s="4" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A151" s="6" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A153" s="6" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A154" s="4" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B154" s="3" t="s">
         <v>16</v>
@@ -3747,7 +3744,7 @@
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A155" s="6" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B155" s="5" t="s">
         <v>16</v>
@@ -3755,7 +3752,7 @@
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A156" s="4" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>16</v>
@@ -3763,7 +3760,7 @@
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A157" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B157" s="5" t="s">
         <v>16</v>
@@ -3771,7 +3768,7 @@
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A158" s="4" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B158" s="3" t="s">
         <v>16</v>
@@ -3779,7 +3776,7 @@
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A159" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B159" s="5" t="s">
         <v>16</v>
@@ -3787,7 +3784,7 @@
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A160" s="4" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>16</v>
@@ -3795,7 +3792,7 @@
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A161" s="6" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B161" s="5" t="s">
         <v>16</v>
@@ -3803,7 +3800,7 @@
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B162" s="3" t="s">
         <v>16</v>
@@ -3811,7 +3808,7 @@
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A163" s="6" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B163" s="5" t="s">
         <v>16</v>
@@ -3819,7 +3816,7 @@
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A164" s="4" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>16</v>
@@ -3827,7 +3824,7 @@
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A165" s="6" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B165" s="5" t="s">
         <v>16</v>
@@ -3835,7 +3832,7 @@
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A166" s="4" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>16</v>
@@ -3843,7 +3840,7 @@
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A167" s="6" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B167" s="5" t="s">
         <v>16</v>
@@ -3851,7 +3848,7 @@
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A168" s="4" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B168" s="3" t="s">
         <v>16</v>
@@ -3859,7 +3856,7 @@
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A169" s="6" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B169" s="5" t="s">
         <v>16</v>
@@ -3867,7 +3864,7 @@
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A170" s="4" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B170" s="3" t="s">
         <v>16</v>
@@ -3875,7 +3872,7 @@
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A171" s="6" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B171" s="5" t="s">
         <v>16</v>
@@ -3883,7 +3880,7 @@
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A172" s="4" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B172" s="3" t="s">
         <v>16</v>
@@ -3891,7 +3888,7 @@
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A173" s="6" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B173" s="5" t="s">
         <v>16</v>
@@ -3899,7 +3896,7 @@
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A174" s="4" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B174" s="3" t="s">
         <v>16</v>
@@ -3907,7 +3904,7 @@
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A175" s="6" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B175" s="5" t="s">
         <v>16</v>
@@ -3915,7 +3912,7 @@
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A176" s="4" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>16</v>
@@ -3923,7 +3920,7 @@
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A177" s="6" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B177" s="5" t="s">
         <v>16</v>
@@ -3931,7 +3928,7 @@
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A178" s="4" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>16</v>
@@ -3939,7 +3936,7 @@
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B179" s="5" t="s">
         <v>16</v>
@@ -3947,7 +3944,7 @@
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A180" s="4" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>16</v>
@@ -3955,7 +3952,7 @@
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A181" s="6" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B181" s="5" t="s">
         <v>16</v>
@@ -3963,7 +3960,7 @@
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A182" s="4" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>16</v>
@@ -3971,7 +3968,7 @@
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A183" s="6" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B183" s="5" t="s">
         <v>16</v>
@@ -3979,7 +3976,7 @@
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A184" s="4" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>16</v>
@@ -3987,7 +3984,7 @@
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A185" s="6" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B185" s="5" t="s">
         <v>16</v>
@@ -3995,7 +3992,7 @@
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A186" s="4" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>16</v>
@@ -4003,7 +4000,7 @@
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A187" s="6" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B187" s="5" t="s">
         <v>16</v>
@@ -4011,7 +4008,7 @@
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A188" s="4" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B188" s="3" t="s">
         <v>16</v>
@@ -4019,7 +4016,7 @@
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A189" s="6" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B189" s="5" t="s">
         <v>16</v>
@@ -4027,7 +4024,7 @@
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A190" s="4" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>16</v>
@@ -4035,7 +4032,7 @@
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A191" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B191" s="5" t="s">
         <v>16</v>
@@ -4043,7 +4040,7 @@
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A192" s="4" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B192" s="3" t="s">
         <v>16</v>
@@ -4051,7 +4048,7 @@
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A193" s="6" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B193" s="5" t="s">
         <v>16</v>
@@ -4059,7 +4056,7 @@
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A194" s="4" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B194" s="3" t="s">
         <v>16</v>
@@ -4067,7 +4064,7 @@
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A195" s="6" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B195" s="5" t="s">
         <v>16</v>
@@ -4075,7 +4072,7 @@
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A196" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B196" s="3" t="s">
         <v>16</v>
@@ -4083,7 +4080,7 @@
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A197" s="6" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B197" s="5" t="s">
         <v>16</v>
@@ -4091,7 +4088,7 @@
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A198" s="4" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B198" s="3" t="s">
         <v>16</v>
@@ -4099,7 +4096,7 @@
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A199" s="6" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B199" s="5" t="s">
         <v>16</v>
@@ -4107,7 +4104,7 @@
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A200" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B200" s="3" t="s">
         <v>16</v>
@@ -4115,7 +4112,7 @@
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A201" s="6" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B201" s="5" t="s">
         <v>16</v>
@@ -4123,7 +4120,7 @@
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A202" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B202" s="3" t="s">
         <v>16</v>
@@ -4131,7 +4128,7 @@
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A203" s="6" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B203" s="5" t="s">
         <v>16</v>
@@ -4139,7 +4136,7 @@
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A204" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B204" s="3" t="s">
         <v>16</v>
@@ -4147,7 +4144,7 @@
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A205" s="6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B205" s="5" t="s">
         <v>16</v>
@@ -4155,7 +4152,7 @@
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A206" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B206" s="3" t="s">
         <v>16</v>
@@ -4163,15 +4160,15 @@
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A207" s="6" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B207" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A208" s="4" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B208" s="3" t="s">
         <v>16</v>
@@ -4179,7 +4176,7 @@
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A209" s="6" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B209" s="5" t="s">
         <v>16</v>
@@ -4187,7 +4184,7 @@
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A210" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B210" s="3" t="s">
         <v>16</v>
@@ -4195,7 +4192,7 @@
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A211" s="6" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B211" s="5" t="s">
         <v>16</v>
@@ -4203,7 +4200,7 @@
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A212" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B212" s="3" t="s">
         <v>16</v>
@@ -4211,7 +4208,7 @@
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A213" s="6" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B213" s="5" t="s">
         <v>16</v>
@@ -4219,7 +4216,7 @@
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A214" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B214" s="3" t="s">
         <v>16</v>
@@ -4227,7 +4224,7 @@
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A215" s="6" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B215" s="5" t="s">
         <v>16</v>
@@ -4235,7 +4232,7 @@
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A216" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B216" s="3" t="s">
         <v>16</v>
@@ -4243,7 +4240,7 @@
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A217" s="6" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B217" s="5" t="s">
         <v>16</v>
@@ -4251,7 +4248,7 @@
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A218" s="4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B218" s="3" t="s">
         <v>16</v>
@@ -4259,399 +4256,399 @@
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A219" s="6" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A220" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B220" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A221" s="6" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B221" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A222" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B222" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A223" s="6" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B223" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A224" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A225" s="6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B225" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A226" s="4" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B226" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A227" s="6" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A228" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A229" s="6" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A230" s="4" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B230" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A231" s="6" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B231" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A232" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B232" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A233" s="6" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B233" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A234" s="4" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B234" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A235" s="6" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B235" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A236" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B236" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A237" s="6" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B237" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A238" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B238" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A239" s="6" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B239" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A240" s="4" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B240" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A241" s="6" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A242" s="4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B242" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A243" s="6" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B243" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A244" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B244" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A245" s="6" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B245" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A246" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B246" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A247" s="6" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A248" s="4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B248" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A249" s="6" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B249" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A250" s="4" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B250" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A251" s="6" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B251" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A252" s="4" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B252" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A253" s="6" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B253" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A254" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B254" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A255" s="6" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A256" s="4" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B256" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A257" s="6" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B257" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A258" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B258" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A259" s="6" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A260" s="4" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B260" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A261" s="6" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B261" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A262" s="4" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B262" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A263" s="6" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B263" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A264" s="4" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B264" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A265" s="6" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B265" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A266" s="4" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A267" s="6" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B267" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A268" s="4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B268" s="3" t="s">
         <v>16</v>
@@ -4659,7 +4656,7 @@
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A269" s="6" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B269" s="5" t="s">
         <v>16</v>
@@ -4667,159 +4664,159 @@
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A270" s="4" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B270" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A271" s="6" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B271" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A272" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B272" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A273" s="6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B273" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A274" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B274" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A275" s="6" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B275" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A276" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B276" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A277" s="6" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A278" s="4" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B278" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A279" s="6" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B279" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A280" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B280" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A281" s="6" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B281" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A282" s="4" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B282" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A283" s="6" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B283" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A284" s="4" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A285" s="6" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B285" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A286" s="4" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B286" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="287" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A287" s="6" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B287" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A288" s="4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B288" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="289" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A289" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B289" s="5" t="s">
         <v>16</v>
@@ -4827,7 +4824,7 @@
     </row>
     <row r="290" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A290" s="4" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B290" s="3" t="s">
         <v>16</v>
@@ -4835,7 +4832,7 @@
     </row>
     <row r="291" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A291" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B291" s="5" t="s">
         <v>16</v>
@@ -4843,7 +4840,7 @@
     </row>
     <row r="292" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A292" s="4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B292" s="3" t="s">
         <v>16</v>
@@ -4851,7 +4848,7 @@
     </row>
     <row r="293" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A293" s="6" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B293" s="5" t="s">
         <v>16</v>
@@ -4859,7 +4856,7 @@
     </row>
     <row r="294" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A294" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B294" s="3" t="s">
         <v>16</v>
@@ -4867,7 +4864,7 @@
     </row>
     <row r="295" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A295" s="6" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B295" s="5" t="s">
         <v>16</v>
@@ -4875,7 +4872,7 @@
     </row>
     <row r="296" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A296" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B296" s="3" t="s">
         <v>16</v>
@@ -4883,7 +4880,7 @@
     </row>
     <row r="297" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A297" s="6" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B297" s="5" t="s">
         <v>16</v>
@@ -4891,66 +4888,66 @@
     </row>
     <row r="298" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A298" s="4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B298" s="3" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="299" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A299" s="6" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B299" s="5" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="300" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A300" s="4" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B300" s="3" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="301" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A301" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B301" s="5" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="302" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A302" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B302" s="3" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A303" s="6" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B303" s="5" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="304" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A304" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B304" s="3" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="305" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A305" s="6" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B305" s="5" t="s">
-        <v>354</v>
+        <v>374</v>
       </c>
     </row>
     <row r="306" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>